<commit_message>
fix: align workbook review status colors
</commit_message>
<xml_diff>
--- a/frontend/public/template-files/monthly-financial-statement-review-template.xlsx
+++ b/frontend/public/template-files/monthly-financial-statement-review-template.xlsx
@@ -511,21 +511,21 @@
   <dxfs count="3">
     <dxf>
       <font>
+        <color rgb="FFD97706"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFEF3C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FFDC2626"/>
       </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFEE2E2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFD97706"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFEF3C7"/>
         </patternFill>
       </fill>
     </dxf>

</xml_diff>